<commit_message>
Update Barley Traits set preharvest sprouting as numerical to support fractional values
</commit_message>
<xml_diff>
--- a/ontology/hordeum-props.xlsx
+++ b/ontology/hordeum-props.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="360">
   <si>
     <t>trait_name</t>
   </si>
@@ -985,18 +985,12 @@
     <t>Colorimeter L* - untreated - parameter value</t>
   </si>
   <si>
-    <t>0/100</t>
-  </si>
-  <si>
     <t>TRAIT: Colorimeter L* parameter ::: METHOD: Colorimeter parameter value - untreated - Computation ::: SCALE: Colorimeter L* parameter value</t>
   </si>
   <si>
     <t>Colorimeter a* - untreated - parameter value</t>
   </si>
   <si>
-    <t>-90/90</t>
-  </si>
-  <si>
     <t>TRAIT: Colorimeter a* parameter ::: METHOD: Colorimeter parameter value - untreated - Computation ::: SCALE: Colorimeter a* parameter value</t>
   </si>
   <si>
@@ -1037,9 +1031,6 @@
   </si>
   <si>
     <t>Wort pH - pH</t>
-  </si>
-  <si>
-    <t>0/14</t>
   </si>
   <si>
     <t>TRAIT: Wort pH ::: METHOD: Wort pH - Measurement ::: SCALE: pH</t>
@@ -3151,10 +3142,13 @@
         <v>312</v>
       </c>
       <c r="B146" t="s">
-        <v>36</v>
-      </c>
-      <c r="F146" t="s">
-        <v>77</v>
+        <v>9</v>
+      </c>
+      <c r="D146">
+        <v>0</v>
+      </c>
+      <c r="E146">
+        <v>9</v>
       </c>
       <c r="G146" t="s">
         <v>313</v>
@@ -3206,227 +3200,203 @@
       <c r="B150" t="s">
         <v>9</v>
       </c>
-      <c r="F150" t="s">
+      <c r="G150" t="s">
         <v>323</v>
-      </c>
-      <c r="G150" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="151" spans="1:7">
       <c r="A151" t="s">
+        <v>324</v>
+      </c>
+      <c r="B151" t="s">
+        <v>9</v>
+      </c>
+      <c r="G151" t="s">
         <v>325</v>
-      </c>
-      <c r="B151" t="s">
-        <v>9</v>
-      </c>
-      <c r="F151" t="s">
-        <v>326</v>
-      </c>
-      <c r="G151" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="152" spans="1:7">
       <c r="A152" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B152" t="s">
         <v>9</v>
       </c>
-      <c r="F152" t="s">
-        <v>326</v>
-      </c>
       <c r="G152" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="153" spans="1:7">
       <c r="A153" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B153" t="s">
         <v>9</v>
       </c>
-      <c r="F153" t="s">
-        <v>323</v>
-      </c>
       <c r="G153" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="154" spans="1:7">
       <c r="A154" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B154" t="s">
         <v>9</v>
       </c>
-      <c r="F154" t="s">
-        <v>326</v>
-      </c>
       <c r="G154" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="155" spans="1:7">
       <c r="A155" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B155" t="s">
         <v>9</v>
       </c>
-      <c r="F155" t="s">
-        <v>326</v>
-      </c>
       <c r="G155" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="156" spans="1:7">
       <c r="A156" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B156" t="s">
         <v>9</v>
       </c>
       <c r="G156" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="157" spans="1:7">
       <c r="A157" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B157" t="s">
         <v>9</v>
       </c>
       <c r="G157" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="158" spans="1:7">
       <c r="A158" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B158" t="s">
         <v>9</v>
       </c>
-      <c r="F158" t="s">
-        <v>341</v>
-      </c>
       <c r="G158" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="159" spans="1:7">
       <c r="A159" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B159" t="s">
         <v>9</v>
       </c>
       <c r="G159" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="160" spans="1:7">
       <c r="A160" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B160" t="s">
         <v>9</v>
       </c>
       <c r="G160" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="161" spans="1:7">
       <c r="A161" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B161" t="s">
         <v>9</v>
       </c>
       <c r="G161" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="162" spans="1:7">
       <c r="A162" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B162" t="s">
         <v>9</v>
       </c>
       <c r="G162" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="163" spans="1:7">
       <c r="A163" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B163" t="s">
         <v>9</v>
       </c>
       <c r="G163" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="164" spans="1:7">
       <c r="A164" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B164" t="s">
         <v>9</v>
       </c>
       <c r="G164" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="165" spans="1:7">
       <c r="A165" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B165" t="s">
         <v>9</v>
       </c>
       <c r="G165" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="166" spans="1:7">
       <c r="A166" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B166" t="s">
         <v>9</v>
       </c>
       <c r="G166" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="167" spans="1:7">
       <c r="A167" t="s">
-        <v>359</v>
-      </c>
-      <c r="F167" t="s">
-        <v>37</v>
+        <v>356</v>
       </c>
       <c r="G167" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="168" spans="1:7">
       <c r="A168" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="B168" t="s">
         <v>9</v>
       </c>
       <c r="G168" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>